<commit_message>
feat(F-NAR-019): TREE-COL-016 passe agent après apply
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-COL-016.xlsx
+++ b/stories/arbres/TREE-COL-016.xlsx
@@ -3090,17 +3090,17 @@
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Victorina installe l'ours brun sur ses genoux. L'ours est lourd, et sent le placard. On fait comme la dernière page, on ne bouge pas. Maman ferme le livre, sans le claquer. Le temps passe, un peu trop long pour les pieds. Victorina ouvre la bouche, puis la referme. Regarde, il a trouvé l'angle sec tout seul. L'oiseau se secoue au-dessus du tapis, derrière le verre. Votre silence lui a laissé de la place.</t>
+          <t>Victorina installe l'ours brun sur ses genoux. L'ours est lourd, et sent le placard. On fait comme la dernière page, on ne bouge pas. Maman ferme le livre, sans le claquer. Le temps passe, un peu trop long pour les pieds. Victorina ouvre la bouche, puis la referme. Regarde, il a trouvé l'angle sec tout seul. L'oiseau se secoue au-dessus du tapis, derrière le verre. Ce silence lui a laissé de la place.</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Victorina installe &lt;emphasis level="moderate"&gt;l'ours&lt;/emphasis&gt; brun sur ses genoux. L'ours est lourd, et sent le placard. On fait comme la dernière page, on ne bouge pas. Maman ferme le livre, sans le claquer. Le temps passe, un peu trop long pour les pieds. Victorina ouvre la bouche, puis la referme. Regarde, il a trouvé l'angle sec tout seul. L'oiseau se secoue au-dessus du tapis, derrière le verre. Votre silence lui a laissé de la place.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Victorina installe &lt;emphasis level="moderate"&gt;l'ours&lt;/emphasis&gt; brun sur ses genoux. L'ours est lourd, et sent le placard. On fait comme la dernière page, on ne bouge pas. Maman ferme le livre, sans le claquer. Le temps passe, un peu trop long pour les pieds. Victorina ouvre la bouche, puis la referme. Regarde, il a trouvé l'angle sec tout seul. L'oiseau se secoue au-dessus du tapis, derrière le verre. Ce silence lui a laissé de la place.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>Victorina installe &lt;emphasis&gt;l'ours&lt;/emphasis&gt; brun sur ses genoux. L'ours est lourd, et sent le placard. On fait comme la dernière page, on ne bouge pas. Maman ferme le livre, sans le claquer. Le temps passe, un peu trop long pour les pieds. Victorina ouvre la bouche, puis la referme. Regarde, il a trouvé l'angle sec tout seul. L'oiseau se secoue au-dessus du tapis, derrière le verre. Votre silence lui a laissé de la place. [pause]</t>
+          <t>Victorina installe &lt;emphasis&gt;l'ours&lt;/emphasis&gt; brun sur ses genoux. L'ours est lourd, et sent le placard. On fait comme la dernière page, on ne bouge pas. Maman ferme le livre, sans le claquer. Le temps passe, un peu trop long pour les pieds. Victorina ouvre la bouche, puis la referme. Regarde, il a trouvé l'angle sec tout seul. L'oiseau se secoue au-dessus du tapis, derrière le verre. Ce silence lui a laissé de la place. [pause]</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr"/>
@@ -3242,7 +3242,7 @@
 narrateur|Victorina ouvre la bouche, puis la referme.
 papa|Regarde, il a trouvé l'angle sec tout seul.
 narrateur|L'oiseau se secoue au-dessus du tapis, derrière le verre.
-maman|Votre silence lui a laissé de la place.</t>
+maman|Ce silence lui a laissé de la place.</t>
         </is>
       </c>
       <c r="AX12" t="inlineStr">
@@ -13483,17 +13483,17 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>L'ours est chaud contre le verre froid. Victorina s'accroupit, le livre fermé sur ses genoux. On ne parle plus, on le laisse choisir. L'oiseau quitte le filet d'eau, pas à pas. Il se secoue si près que la vitre s'embue. On n'a rien forcé, et il a trouvé. L'ours garde une petite buée sur le nez.</t>
+          <t>L'ours est chaud contre le verre froid. Victorina s'accroupit, le livre fermé sur ses genoux. On ne parle plus, on le laisse choisir. L'oiseau quitte le filet d'eau, pas à pas. Il se secoue si près que la vitre s'embue. On a attendu, et il a trouvé son angle. L'ours garde une petite buée sur le nez.</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;L'ours est chaud contre le verre froid. Victorina s'accroupit, le livre fermé sur ses genoux. On ne parle plus, on le laisse choisir. L'oiseau quitte le filet d'eau, pas à pas. Il se secoue si près que la vitre s'embue. On n'a rien forcé, et il a trouvé. L'ours garde une petite buée sur le nez.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;L'ours est chaud contre le verre froid. Victorina s'accroupit, le livre fermé sur ses genoux. On ne parle plus, on le laisse choisir. L'oiseau quitte le filet d'eau, pas à pas. Il se secoue si près que la vitre s'embue. On a attendu, et il a trouvé son angle. L'ours garde une petite buée sur le nez.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G68" s="2" t="inlineStr">
         <is>
-          <t>L'ours est chaud contre le verre froid. Victorina s'accroupit, le livre fermé sur ses genoux. On ne parle plus, on le laisse choisir. L'oiseau quitte le filet d'eau, pas à pas. Il se secoue si près que la vitre s'embue. On n'a rien forcé, et il a trouvé. L'ours garde une petite buée sur le nez. [pause]</t>
+          <t>L'ours est chaud contre le verre froid. Victorina s'accroupit, le livre fermé sur ses genoux. On ne parle plus, on le laisse choisir. L'oiseau quitte le filet d'eau, pas à pas. Il se secoue si près que la vitre s'embue. On a attendu, et il a trouvé son angle. L'ours garde une petite buée sur le nez. [pause]</t>
         </is>
       </c>
       <c r="H68" s="2" t="inlineStr"/>
@@ -13632,7 +13632,7 @@
 enfant-f|On ne parle plus, on le laisse choisir.
 narrateur|L'oiseau quitte le filet d'eau, pas à pas.
 narrateur|Il se secoue si près que la vitre s'embue.
-papa|On n'a rien forcé, et il a trouvé.
+papa|On a attendu, et il a trouvé son angle.
 narrateur|L'ours garde une petite buée sur le nez.</t>
         </is>
       </c>
@@ -14215,17 +14215,17 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>Face à la vitre, papa chante tout bas. Les gouttes suivent, puis se taisent. Je veux le refrain maintenant ! Sa voix recouvre le dernier mot de papa. L'oiseau recule d'un pas, méfiant. Laisse-moi finir, ensuite c'est toi. Victorina serre ses poings, puis les ouvre. Elle attend le point, et elle pose sa note. L'oiseau avance, et glisse un cri dans le trou. Il chante avec vous, chacun son trou. On ne lui marche plus sur le bec.</t>
+          <t>Face à la vitre, papa chante tout bas. Les gouttes suivent, puis se taisent. Je veux le refrain maintenant ! Sa voix recouvre le dernier mot de papa. L'oiseau recule d'un pas, méfiant. Laisse-moi finir, ensuite c'est toi. Victorina serre ses poings, puis les ouvre. Elle attend le point, et elle pose sa note. L'oiseau avance, et glisse un cri dans le trou. Il chante avec vous, chacun son trou. Cette fois, on lui laisse son cri.</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Face à la vitre, papa chante tout bas. Les gouttes suivent, puis se taisent. Je veux le refrain maintenant ! Sa voix recouvre le dernier mot de papa. L'&lt;emphasis level="moderate"&gt;oiseau&lt;/emphasis&gt; recule d'un pas, méfiant. Laisse-moi finir, ensuite c'est toi. Victorina serre ses poings, puis les ouvre. Elle attend le point, et elle pose sa note. L'oiseau avance, et glisse un cri dans le trou. Il chante avec vous, chacun son trou. On ne lui marche plus sur le bec.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="-2st"&gt;Face à la vitre, papa chante tout bas. Les gouttes suivent, puis se taisent. Je veux le refrain maintenant ! Sa voix recouvre le dernier mot de papa. L'&lt;emphasis level="moderate"&gt;oiseau&lt;/emphasis&gt; recule d'un pas, méfiant. Laisse-moi finir, ensuite c'est toi. Victorina serre ses poings, puis les ouvre. Elle attend le point, et elle pose sa note. L'oiseau avance, et glisse un cri dans le trou. Il chante avec vous, chacun son trou. Cette fois, on lui laisse son cri.&lt;/prosody&gt;&lt;break time="520ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G72" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;Face à la vitre, papa chante tout bas. Les gouttes suivent, puis se taisent. Je veux le refrain maintenant ! Sa voix recouvre le dernier mot de papa. L'&lt;emphasis&gt;oiseau&lt;/emphasis&gt; recule d'un pas, méfiant. Laisse-moi finir, ensuite c'est toi. Victorina serre ses poings, puis les ouvre. Elle attend le point, et elle pose sa note. L'oiseau avance, et glisse un cri dans le trou. Il chante avec vous, chacun son trou. On ne lui marche plus sur le bec.&lt;/low-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;Face à la vitre, papa chante tout bas. Les gouttes suivent, puis se taisent. Je veux le refrain maintenant ! Sa voix recouvre le dernier mot de papa. L'&lt;emphasis&gt;oiseau&lt;/emphasis&gt; recule d'un pas, méfiant. Laisse-moi finir, ensuite c'est toi. Victorina serre ses poings, puis les ouvre. Elle attend le point, et elle pose sa note. L'oiseau avance, et glisse un cri dans le trou. Il chante avec vous, chacun son trou. Cette fois, on lui laisse son cri.&lt;/low-pitch&gt; [pause]</t>
         </is>
       </c>
       <c r="H72" s="2" t="inlineStr"/>
@@ -14373,7 +14373,7 @@
 narrateur|Elle attend le point, et elle pose sa note.
 narrateur|L'oiseau avance, et glisse un cri dans le trou.
 maman|Il chante avec vous, chacun son trou.
-enfant-f|On ne lui marche plus sur le bec.</t>
+enfant-f|Cette fois, on lui laisse son cri.</t>
         </is>
       </c>
       <c r="AX72" t="inlineStr">
@@ -17177,7 +17177,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A16"/>
+  <dimension ref="A1:A17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -17290,6 +17290,13 @@
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>